<commit_message>
prepare final demo data and align delivery artifacts
</commit_message>
<xml_diff>
--- a/output/backlog/GoalZone_Backlog_Final_Code_First_2026-07-26.xlsx
+++ b/output/backlog/GoalZone_Backlog_Final_Code_First_2026-07-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="R17c7ec1a52aa4c0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contribution" sheetId="2" r:id="Re81c922359d441c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" r:id="R1960cd5393224994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contribution" sheetId="2" r:id="R4a1fc33643974e31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2507,7 +2507,7 @@
         <x:v>Ask availability assistant</x:v>
       </x:c>
       <x:c r="F63" s="8" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G63" s="11" t="n">
         <x:v>46152</x:v>
@@ -2519,7 +2519,7 @@
         <x:v>A signed-in customer asks Gemini to interpret a natural-language field request; all displayed availability remains grounded in live GoalZone data.</x:v>
       </x:c>
       <x:c r="J63" s="6" t="str">
-        <x:v>Implementation is present and uses Gemini 3.6 Flash for criteria extraction and concise wording. Deployment remains Deferred until GEMINI_API_KEY is configured and one external smoke test passes; missing configuration correctly returns HTTP 503.</x:v>
+        <x:v>Implemented, externally verified, and shippable. Gemini 3.6 Flash extracts constrained search criteria and phrases a concise answer, while live GoalZone field, slot, price, membership, and promotion data remain authoritative. GEMINI_API_KEY and GEMINI_MODEL are runtime deployment configuration, not unfinished backlog scope; UC-63 deterministic filters remain available independently.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="39" customHeight="1">
@@ -3533,7 +3533,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2276825ec649a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d7ee5e555fc4a9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4628,7 +4628,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24198ac8278d4413"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc83f2ed68014489f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>